<commit_message>
Add Excel stopwatch, Google Sheets Apps Script, and setup helper.
Judges get .xlsm macro buttons for Log Run; Google Sheets users install Apps Script with one-click setupLogRunSheet for formulas and stopwatch menu.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/LKS2026-Penilaian-Juri-CONTOH.xlsx
+++ b/templates/LKS2026-Penilaian-Juri-CONTOH.xlsx
@@ -24,10 +24,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="hh:mm:ss"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,8 +80,18 @@
       <i val="1"/>
       <color rgb="00C00000"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00404040"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -102,6 +113,16 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F4FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -121,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -151,7 +172,19 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="46" fontId="11" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="46" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -519,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -650,69 +683,76 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2. Modul A/B/C: isi skor Juri 1-3 (0-3). Skor otomatis.</t>
+          <t xml:space="preserve">   Disarankan: LKS2026-Penilaian-Juri.xlsm (stopwatch Log Run — Enable Macro).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>3. Modul B: isi Tepat Waktu (1/0) di G4.</t>
+          <t>2. Modul A/B/C: isi skor Juri 1-3 (0-3). Skor otomatis.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>4. UNDIAN KUBUS (isi DULU sebelum Modul E):</t>
+          <t>3. Modul B: isi Tepat Waktu (1/0) di G4.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">   a. Baris 24 (kuning): warna marker Merah/Hijau/Biru per slot.</t>
+          <t>4. UNDIAN KUBUS (isi DULU sebelum Modul E):</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">   b. Baris 28–36: kolom A = ID kubus | E = Rak/Stand | F = Slot.</t>
+          <t xml:space="preserve">   a. Baris 24 (kuning): warna marker Merah/Hijau/Biru per slot.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>5. MODUL E: kolom B-G otomatis. Juri isi kolom H (Hasil Run 1/0) saja.</t>
+          <t xml:space="preserve">   b. Baris 28–36: kolom A = ID kubus | E = Rak/Stand | F = Slot.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">   OK Awal = posisi sudah benar sebelum run | Hasil Run = sukses setelah run.</t>
+          <t>5. MODUL E: kolom B-G otomatis. Juri isi kolom H (Hasil Run 1/0) saja.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>6. Log Run Otonom: checklist SIAP/START + kronologi.</t>
+          <t xml:space="preserve">   OK Awal = posisi sudah benar sebelum run | Hasil Run = sukses setelah run.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>6. Log Run Otonom: tombol stopwatch SIAP/START/SELESAI (.xlsm) + checklist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>7. Rekapitulasi: total otomatis. Input ke CIS (Chief Expert).</t>
         </is>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Sheet: Panduan | Modul A-E | Undian Kubus | Log Run | Rekapitulasi</t>
         </is>
@@ -3574,14 +3614,14 @@
           <t>Waktu START:</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>08:42</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>PETUNJUK: Isi sheet Undian Kubus dulu — baris 24 (warna marker, baris kuning), kolom A baris 28–36 (ID kubus), E (Rak/Stand), F (Slot). Kolom di bawah terisi otomatis.</t>
         </is>
@@ -4084,7 +4124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4095,6 +4135,9 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4160,10 +4203,15 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="28" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>DATA RUN</t>
+        </is>
+      </c>
+      <c r="J6" s="17" t="inlineStr">
+        <is>
+          <t>STOPWATCH RUN — klik tombol di bawah (file .xlsm, Enable Macro)</t>
         </is>
       </c>
     </row>
@@ -4193,6 +4241,15 @@
           <t>Trial</t>
         </is>
       </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>Durasi live (F9):</t>
+        </is>
+      </c>
+      <c r="K7" s="18">
+        <f>IF(E8="","",IF(H8&lt;&gt;"",H8-E8,NOW()-TODAY()-E8))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -4200,15 +4257,39 @@
           <t>Waktu SIAP:</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08:40:00</t>
+        </is>
+      </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Waktu START:</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>08:42:00</t>
+        </is>
+      </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
           <t>Waktu Selesai:</t>
         </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>08:55:00</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>Durasi final:</t>
+        </is>
+      </c>
+      <c r="K8" s="19">
+        <f>IF(AND(E8&lt;&gt;"",H8&lt;&gt;""),H8-E8,"")</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -4225,6 +4306,22 @@
       <c r="G9" s="7" t="inlineStr">
         <is>
           <t>Retry No:</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>Menit:</t>
+        </is>
+      </c>
+      <c r="K9" s="20">
+        <f>IF(K8="","",ROUND(K8*24*60,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="J10" s="21" t="inlineStr">
+        <is>
+          <t>Tanpa macro (.xlsx): Ctrl+Shift+: untuk waktu | tekan F9 saat run untuk refresh durasi live. Disarankan .xlsm + tombol ▶ SIAP ▶ START ■ SELESAI (Enable Macro).</t>
         </is>
       </c>
     </row>
@@ -4464,9 +4561,11 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
+    <mergeCell ref="J6:L6"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="J10:L10"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>

</xml_diff>